<commit_message>
finish analysis, graphs and tables -- 1st round
</commit_message>
<xml_diff>
--- a/analysis_ready_data/port_blakely/Port Blakely Cedar Info.xlsx
+++ b/analysis_ready_data/port_blakely/Port Blakely Cedar Info.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdixon\Documents\PhD\browse_study\Browse_analysis\analysis_ready_data\port_blakely\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0540E9D2-D301-4A03-A354-CB941DE51807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{035085C1-41E9-4FB4-A623-A7E957159716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="624" yWindow="60" windowWidth="19884" windowHeight="11604" firstSheet="1" activeTab="3" xr2:uid="{279772AA-D708-4943-A4E5-531146DFFF78}"/>
+    <workbookView xWindow="-16290" yWindow="-4830" windowWidth="15465" windowHeight="15585" activeTab="3" xr2:uid="{279772AA-D708-4943-A4E5-531146DFFF78}"/>
   </bookViews>
   <sheets>
     <sheet name="reformatted" sheetId="5" r:id="rId1"/>
-    <sheet name="raw_data" sheetId="6" r:id="rId2"/>
-    <sheet name="Silvi History Punky Root" sheetId="1" r:id="rId3"/>
-    <sheet name="12year_crz_Punky Root" sheetId="2" r:id="rId4"/>
-    <sheet name="Silvi History Rotten Bull" sheetId="4" r:id="rId5"/>
+    <sheet name="punky_root_raw_data" sheetId="7" r:id="rId2"/>
+    <sheet name="raw_data" sheetId="6" r:id="rId3"/>
+    <sheet name="Silvi History Punky Root" sheetId="1" r:id="rId4"/>
+    <sheet name="12year_crz_Punky Root" sheetId="2" r:id="rId5"/>
+    <sheet name="Silvi History Rotten Bull" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6292" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6362" uniqueCount="210">
   <si>
     <r>
       <t xml:space="preserve">Location: </t>
@@ -654,6 +655,36 @@
   <si>
     <t>Dead</t>
   </si>
+  <si>
+    <t>Stand</t>
+  </si>
+  <si>
+    <t>Plot</t>
+  </si>
+  <si>
+    <t>Tree</t>
+  </si>
+  <si>
+    <t>Spc</t>
+  </si>
+  <si>
+    <t>Cnt</t>
+  </si>
+  <si>
+    <t>Crown Height</t>
+  </si>
+  <si>
+    <t>Broken Height</t>
+  </si>
+  <si>
+    <t>0111N03E032874_22</t>
+  </si>
+  <si>
+    <t>in</t>
+  </si>
+  <si>
+    <t>out</t>
+  </si>
 </sst>
 </file>
 
@@ -1256,6 +1287,813 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6F31170-D294-47BC-B9D1-D644439797E2}">
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" t="s">
+        <v>204</v>
+      </c>
+      <c r="H1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" t="s">
+        <v>205</v>
+      </c>
+      <c r="J1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>40</v>
+      </c>
+      <c r="F2">
+        <v>3.3</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>19</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>60</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>17</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+      <c r="G4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>207</v>
+      </c>
+      <c r="B5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>40</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>40</v>
+      </c>
+      <c r="F6">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>20</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>40</v>
+      </c>
+      <c r="G7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B8" t="s">
+        <v>208</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>40</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" t="s">
+        <v>208</v>
+      </c>
+      <c r="C9">
+        <v>4</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>60</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>18</v>
+      </c>
+      <c r="I9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B10" t="s">
+        <v>209</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>40</v>
+      </c>
+      <c r="F10">
+        <v>2.5</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>13</v>
+      </c>
+      <c r="I10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
+        <v>40</v>
+      </c>
+      <c r="F11">
+        <v>5.8</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>19</v>
+      </c>
+      <c r="I11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B12" t="s">
+        <v>209</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>40</v>
+      </c>
+      <c r="G12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13" t="s">
+        <v>209</v>
+      </c>
+      <c r="C13">
+        <v>6</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>60</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>15</v>
+      </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>207</v>
+      </c>
+      <c r="B14" t="s">
+        <v>209</v>
+      </c>
+      <c r="C14">
+        <v>6</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14">
+        <v>60</v>
+      </c>
+      <c r="F14">
+        <v>1.6</v>
+      </c>
+      <c r="H14">
+        <v>19</v>
+      </c>
+      <c r="I14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" t="s">
+        <v>209</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>60</v>
+      </c>
+      <c r="G15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" t="s">
+        <v>209</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>4</v>
+      </c>
+      <c r="E16">
+        <v>20</v>
+      </c>
+      <c r="F16">
+        <v>1.2</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>12</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" t="s">
+        <v>209</v>
+      </c>
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>40</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>207</v>
+      </c>
+      <c r="B18" t="s">
+        <v>209</v>
+      </c>
+      <c r="C18">
+        <v>7</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>40</v>
+      </c>
+      <c r="F18">
+        <v>6.9</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>21</v>
+      </c>
+      <c r="I18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" t="s">
+        <v>209</v>
+      </c>
+      <c r="C19">
+        <v>7</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>40</v>
+      </c>
+      <c r="G19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>207</v>
+      </c>
+      <c r="B20" t="s">
+        <v>209</v>
+      </c>
+      <c r="C20">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20">
+        <v>60</v>
+      </c>
+      <c r="G20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21" t="s">
+        <v>209</v>
+      </c>
+      <c r="C21">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>60</v>
+      </c>
+      <c r="F21">
+        <v>1.2</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>16</v>
+      </c>
+      <c r="I21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>207</v>
+      </c>
+      <c r="B22" t="s">
+        <v>209</v>
+      </c>
+      <c r="C22">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>60</v>
+      </c>
+      <c r="F22">
+        <v>1.5</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>16</v>
+      </c>
+      <c r="I22">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>207</v>
+      </c>
+      <c r="B23" t="s">
+        <v>209</v>
+      </c>
+      <c r="C23">
+        <v>8</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23">
+        <v>60</v>
+      </c>
+      <c r="F23">
+        <v>1.2</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>16</v>
+      </c>
+      <c r="I23">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B24" t="s">
+        <v>209</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24">
+        <v>60</v>
+      </c>
+      <c r="G24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>207</v>
+      </c>
+      <c r="B25" t="s">
+        <v>209</v>
+      </c>
+      <c r="C25">
+        <v>8</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25">
+        <v>10</v>
+      </c>
+      <c r="F25">
+        <v>2.4</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>17</v>
+      </c>
+      <c r="I25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>207</v>
+      </c>
+      <c r="B26" t="s">
+        <v>209</v>
+      </c>
+      <c r="C26">
+        <v>8</v>
+      </c>
+      <c r="D26">
+        <v>6</v>
+      </c>
+      <c r="E26">
+        <v>10</v>
+      </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>25</v>
+      </c>
+      <c r="I26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>207</v>
+      </c>
+      <c r="B27" t="s">
+        <v>209</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>7</v>
+      </c>
+      <c r="E27">
+        <v>10</v>
+      </c>
+      <c r="F27">
+        <v>2.1</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>14</v>
+      </c>
+      <c r="I27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>207</v>
+      </c>
+      <c r="B28" t="s">
+        <v>209</v>
+      </c>
+      <c r="C28">
+        <v>8</v>
+      </c>
+      <c r="D28">
+        <v>8</v>
+      </c>
+      <c r="E28">
+        <v>30</v>
+      </c>
+      <c r="F28">
+        <v>1.5</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <v>12</v>
+      </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" t="s">
+        <v>209</v>
+      </c>
+      <c r="C29">
+        <v>8</v>
+      </c>
+      <c r="D29">
+        <v>9</v>
+      </c>
+      <c r="E29">
+        <v>30</v>
+      </c>
+      <c r="F29">
+        <v>1.2</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>8</v>
+      </c>
+      <c r="I29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>207</v>
+      </c>
+      <c r="B30" t="s">
+        <v>209</v>
+      </c>
+      <c r="C30">
+        <v>8</v>
+      </c>
+      <c r="D30">
+        <v>10</v>
+      </c>
+      <c r="E30">
+        <v>30</v>
+      </c>
+      <c r="F30">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>15</v>
+      </c>
+      <c r="I30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>207</v>
+      </c>
+      <c r="B31" t="s">
+        <v>209</v>
+      </c>
+      <c r="C31">
+        <v>8</v>
+      </c>
+      <c r="D31">
+        <v>11</v>
+      </c>
+      <c r="E31">
+        <v>30</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BD8775A-BD07-4CBD-A4B8-CB7E8C5A9627}">
   <dimension ref="A1:C1981"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -23059,7 +23897,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30DF8E99-95DA-46E6-9940-353E6DC83246}">
   <dimension ref="A1:M125"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -23908,7 +24746,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D439A4A-DB3E-4724-B2D7-2B7864D256AF}">
   <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -24534,7 +25372,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97C60041-AD41-4459-8A0C-4F6664081368}">
   <dimension ref="A1:M56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>